<commit_message>
Seleccion y justificacion de dataSets y Preprocesamiento de datos
</commit_message>
<xml_diff>
--- a/Requisitos.xlsx
+++ b/Requisitos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unaledu-my.sharepoint.com/personal/mzueta_unal_edu_co/Documents/2025-02/Intro IA/Practica 2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unaledu-my.sharepoint.com/personal/mzueta_unal_edu_co/Documents/2025-02/Intro IA/Practica 2/practica_2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{5DEF330F-B20D-48E4-BD39-5B1BF5609BEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A2F4850-DF22-42AE-8FCC-86952C6C5ED0}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="8_{5DEF330F-B20D-48E4-BD39-5B1BF5609BEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5842D9D1-B35A-4996-A149-B1AD47F7EBFD}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{C3C9E867-635C-465D-A0EB-854244AC6264}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="33">
   <si>
     <t>Responsable</t>
   </si>
@@ -129,6 +129,12 @@
   </si>
   <si>
     <t>Generar ZIP con PDF, código y video. Subir a Google Classroom con nombre correcto del archivo. Verificar consistencia entre código, video y documento.</t>
+  </si>
+  <si>
+    <t>MANUEL ZULETA ARANGO</t>
+  </si>
+  <si>
+    <t>TODOS</t>
   </si>
 </sst>
 </file>
@@ -227,6 +233,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -579,7 +589,7 @@
     </row>
     <row r="2" spans="1:3" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>4</v>
@@ -590,7 +600,7 @@
     </row>
     <row r="3" spans="1:3" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>6</v>
@@ -689,7 +699,7 @@
     </row>
     <row r="12" spans="1:3" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>27</v>

</xml_diff>

<commit_message>
creacion de graficas y evaluacion de modelos
</commit_message>
<xml_diff>
--- a/Requisitos.xlsx
+++ b/Requisitos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unaledu-my.sharepoint.com/personal/mzueta_unal_edu_co/Documents/2025-02/Intro IA/Practica 2/practica_2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="8_{5DEF330F-B20D-48E4-BD39-5B1BF5609BEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5842D9D1-B35A-4996-A149-B1AD47F7EBFD}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="8_{5DEF330F-B20D-48E4-BD39-5B1BF5609BEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15048981-FBD3-43B1-B37C-5FDF063CABDD}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{C3C9E867-635C-465D-A0EB-854244AC6264}"/>
   </bookViews>
@@ -141,7 +141,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -151,6 +151,14 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -178,7 +186,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -186,6 +194,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -568,7 +577,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6937F141-99F3-41DF-9A3A-86F8916DDB77}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="122.28515625" customWidth="1"/>
@@ -710,7 +719,7 @@
     </row>
     <row r="13" spans="1:3" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>29</v>
@@ -718,6 +727,9 @@
       <c r="C13" s="2" t="s">
         <v>30</v>
       </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
creacion de visualizaciones de modelos supervisados
</commit_message>
<xml_diff>
--- a/Requisitos.xlsx
+++ b/Requisitos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unaledu-my.sharepoint.com/personal/mzueta_unal_edu_co/Documents/2025-02/Intro IA/Practica 2/practica_2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="8_{5DEF330F-B20D-48E4-BD39-5B1BF5609BEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{15048981-FBD3-43B1-B37C-5FDF063CABDD}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="8_{5DEF330F-B20D-48E4-BD39-5B1BF5609BEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3F7C5D18-AD0B-4D94-AB0C-B5BAF3FF7300}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{C3C9E867-635C-465D-A0EB-854244AC6264}"/>
   </bookViews>
@@ -620,7 +620,7 @@
     </row>
     <row r="4" spans="1:3" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>9</v>
@@ -631,7 +631,7 @@
     </row>
     <row r="5" spans="1:3" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>11</v>
@@ -642,7 +642,7 @@
     </row>
     <row r="6" spans="1:3" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>14</v>

</xml_diff>